<commit_message>
Registrar o post de 26/08 como publicado
Grava no arquivo a versao exata que foi ao ar, com a chamada final em
"Comenta aqui", e remove a nota de correcao ja incorporada.

Acrescenta o post ao acompanhamento como serie Extra, para que ele entre na
comparacao junto com os 16 planejados. O plano passa a ser ordenado por data
antes de escrever as linhas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rs5hehAPo3WmcKFkRQTrtS
</commit_message>
<xml_diff>
--- a/analise/acompanhamento.xlsx
+++ b/analise/acompanhamento.xlsx
@@ -523,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
+  <dimension ref="A1:O27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -747,27 +747,27 @@
         <v>2</v>
       </c>
       <c r="B9" s="10">
-        <f>$C$4+2</f>
+        <f>$C$4+1</f>
         <v/>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Qua</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Farinha importada</t>
+          <t>Pala e Pinsa, teglia e contemporânea</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Opinião Impopular</t>
+          <t>Extra</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Card/Reels</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="G9" s="11" t="n"/>
@@ -794,27 +794,27 @@
         <v>3</v>
       </c>
       <c r="B10" s="10">
-        <f>$C$4+4</f>
+        <f>$C$4+2</f>
         <v/>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Criação autoral</t>
+          <t>Farinha importada</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Autoral</t>
+          <t>Opinião Impopular</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Foto</t>
+          <t>Card/Reels</t>
         </is>
       </c>
       <c r="G10" s="11" t="n"/>
@@ -841,27 +841,27 @@
         <v>4</v>
       </c>
       <c r="B11" s="10">
-        <f>$C$4+5</f>
+        <f>$C$4+4</f>
         <v/>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Ponto de véu</t>
+          <t>Criação autoral</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>O Porquê</t>
+          <t>Autoral</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Foto</t>
         </is>
       </c>
       <c r="G11" s="11" t="n"/>
@@ -888,27 +888,27 @@
         <v>5</v>
       </c>
       <c r="B12" s="10">
-        <f>$C$4+7</f>
+        <f>$C$4+5</f>
         <v/>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Ter</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>48h de maturação</t>
+          <t>Ponto de véu</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>O Porquê do Número</t>
+          <t>O Porquê</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Carrossel</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="G12" s="11" t="n"/>
@@ -935,22 +935,22 @@
         <v>6</v>
       </c>
       <c r="B13" s="10">
-        <f>$C$4+9</f>
+        <f>$C$4+7</f>
         <v/>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Ter</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>24h contra 48h</t>
+          <t>48h de maturação</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>Uma Variável</t>
+          <t>O Porquê do Número</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
@@ -982,22 +982,22 @@
         <v>7</v>
       </c>
       <c r="B14" s="10">
-        <f>$C$4+11</f>
+        <f>$C$4+9</f>
         <v/>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Cronograma de produção</t>
+          <t>24h contra 48h</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Bastidores</t>
+          <t>Uma Variável</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
@@ -1029,27 +1029,27 @@
         <v>8</v>
       </c>
       <c r="B15" s="10">
-        <f>$C$4+12</f>
+        <f>$C$4+11</f>
         <v/>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Temperatura da água</t>
+          <t>Cronograma de produção</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>O Porquê</t>
+          <t>Bastidores</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Carrossel</t>
         </is>
       </c>
       <c r="G15" s="11" t="n"/>
@@ -1076,27 +1076,27 @@
         <v>9</v>
       </c>
       <c r="B16" s="10">
-        <f>$C$4+14</f>
+        <f>$C$4+12</f>
         <v/>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Ter</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>W300, força da farinha</t>
+          <t>Temperatura da água</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>O Porquê do Número</t>
+          <t>O Porquê</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>Carrossel</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="G16" s="11" t="n"/>
@@ -1123,27 +1123,27 @@
         <v>10</v>
       </c>
       <c r="B17" s="10">
-        <f>$C$4+16</f>
+        <f>$C$4+14</f>
         <v/>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Ter</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Forno caro</t>
+          <t>W300, força da farinha</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Opinião Impopular</t>
+          <t>O Porquê do Número</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Card/Reels</t>
+          <t>Carrossel</t>
         </is>
       </c>
       <c r="G17" s="11" t="n"/>
@@ -1170,27 +1170,27 @@
         <v>11</v>
       </c>
       <c r="B18" s="10">
-        <f>$C$4+18</f>
+        <f>$C$4+16</f>
         <v/>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>O erro que me custou caro</t>
+          <t>Forno caro</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>O Erro</t>
+          <t>Opinião Impopular</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Card/Reels</t>
         </is>
       </c>
       <c r="G18" s="11" t="n"/>
@@ -1217,22 +1217,22 @@
         <v>12</v>
       </c>
       <c r="B19" s="10">
-        <f>$C$4+19</f>
+        <f>$C$4+18</f>
         <v/>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>Biga contra poolish</t>
+          <t>O erro que me custou caro</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>O Porquê</t>
+          <t>O Erro</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
@@ -1264,27 +1264,27 @@
         <v>13</v>
       </c>
       <c r="B20" s="10">
-        <f>$C$4+21</f>
+        <f>$C$4+19</f>
         <v/>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>Ter</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>450°C no forno</t>
+          <t>Biga contra poolish</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>O Porquê do Número</t>
+          <t>O Porquê</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Carrossel</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="G20" s="11" t="n"/>
@@ -1311,22 +1311,22 @@
         <v>14</v>
       </c>
       <c r="B21" s="10">
-        <f>$C$4+23</f>
+        <f>$C$4+21</f>
         <v/>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Ter</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>60% contra 70%</t>
+          <t>450°C no forno</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Uma Variável</t>
+          <t>O Porquê do Número</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
@@ -1358,22 +1358,22 @@
         <v>15</v>
       </c>
       <c r="B22" s="10">
-        <f>$C$4+25</f>
+        <f>$C$4+23</f>
         <v/>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>Aula, turmas em SP</t>
+          <t>60% contra 70%</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Formação</t>
+          <t>Uma Variável</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
@@ -1405,27 +1405,27 @@
         <v>16</v>
       </c>
       <c r="B23" s="10">
-        <f>$C$4+26</f>
+        <f>$C$4+25</f>
         <v/>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Os 3 números</t>
+          <t>Aula, turmas em SP</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>O Porquê</t>
+          <t>Formação</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Carrossel</t>
         </is>
       </c>
       <c r="G23" s="11" t="n"/>
@@ -1447,62 +1447,109 @@
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="D25" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="9" t="n">
+        <v>17</v>
+      </c>
+      <c r="B24" s="10">
+        <f>$C$4+26</f>
+        <v/>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Dom</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Os 3 números</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>O Porquê</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n"/>
+      <c r="H24" s="11" t="n"/>
+      <c r="I24" s="11" t="n"/>
+      <c r="J24" s="11" t="n"/>
+      <c r="K24" s="11" t="n"/>
+      <c r="L24" s="11" t="n"/>
+      <c r="M24" s="12">
+        <f>IFERROR(H24/G24,"")</f>
+        <v/>
+      </c>
+      <c r="N24" s="12">
+        <f>IFERROR(L24/G24,"")</f>
+        <v/>
+      </c>
+      <c r="O24" s="12">
+        <f>IFERROR(K24/G24,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>MÉDIA DO MÊS</t>
         </is>
       </c>
-      <c r="G25" s="13">
-        <f>IFERROR(AVERAGE(G8:G23),"")</f>
-        <v/>
-      </c>
-      <c r="H25" s="13">
-        <f>IFERROR(AVERAGE(H8:H23),"")</f>
-        <v/>
-      </c>
-      <c r="I25" s="13">
-        <f>IFERROR(AVERAGE(I8:I23),"")</f>
-        <v/>
-      </c>
-      <c r="J25" s="13">
-        <f>IFERROR(AVERAGE(J8:J23),"")</f>
-        <v/>
-      </c>
-      <c r="K25" s="13">
-        <f>IFERROR(AVERAGE(K8:K23),"")</f>
-        <v/>
-      </c>
-      <c r="L25" s="13">
-        <f>IFERROR(AVERAGE(L8:L23),"")</f>
-        <v/>
-      </c>
-      <c r="M25" s="14">
-        <f>IFERROR(AVERAGE(M8:M23),"")</f>
-        <v/>
-      </c>
-      <c r="N25" s="14">
-        <f>IFERROR(AVERAGE(N8:N23),"")</f>
-        <v/>
-      </c>
-      <c r="O25" s="14">
-        <f>IFERROR(AVERAGE(O8:O23),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="D26" s="2" t="inlineStr">
+      <c r="G26" s="13">
+        <f>IFERROR(AVERAGE(G8:G24),"")</f>
+        <v/>
+      </c>
+      <c r="H26" s="13">
+        <f>IFERROR(AVERAGE(H8:H24),"")</f>
+        <v/>
+      </c>
+      <c r="I26" s="13">
+        <f>IFERROR(AVERAGE(I8:I24),"")</f>
+        <v/>
+      </c>
+      <c r="J26" s="13">
+        <f>IFERROR(AVERAGE(J8:J24),"")</f>
+        <v/>
+      </c>
+      <c r="K26" s="13">
+        <f>IFERROR(AVERAGE(K8:K24),"")</f>
+        <v/>
+      </c>
+      <c r="L26" s="13">
+        <f>IFERROR(AVERAGE(L8:L24),"")</f>
+        <v/>
+      </c>
+      <c r="M26" s="14">
+        <f>IFERROR(AVERAGE(M8:M24),"")</f>
+        <v/>
+      </c>
+      <c r="N26" s="14">
+        <f>IFERROR(AVERAGE(N8:N24),"")</f>
+        <v/>
+      </c>
+      <c r="O26" s="14">
+        <f>IFERROR(AVERAGE(O8:O24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Ponto de partida (agosto/26)</t>
         </is>
       </c>
-      <c r="L26" s="2" t="n">
+      <c r="L27" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="N26" s="15" t="n">
+      <c r="N27" s="15" t="n">
         <v>0.003</v>
       </c>
-      <c r="O26" s="5" t="inlineStr">
+      <c r="O27" s="5" t="inlineStr">
         <is>
           <t>← a meta é dobrar esta coluna</t>
         </is>
@@ -1519,7 +1566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1583,23 +1630,23 @@
         </is>
       </c>
       <c r="B5" s="17">
-        <f>COUNTIF(Acompanhamento!$E$8:$E$23,A5)</f>
+        <f>COUNTIF(Acompanhamento!$E$8:$E$24,A5)</f>
         <v/>
       </c>
       <c r="C5" s="18">
-        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A5),"")</f>
+        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A5),"")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$23,Acompanhamento!$E$8:$E$23,A5)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A5),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$24,Acompanhamento!$E$8:$E$24,A5)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A5),"")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A5)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A5),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A5)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A5),"")</f>
         <v/>
       </c>
       <c r="F5" s="18">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A5),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A5),"")</f>
         <v/>
       </c>
     </row>
@@ -1610,23 +1657,23 @@
         </is>
       </c>
       <c r="B6" s="17">
-        <f>COUNTIF(Acompanhamento!$E$8:$E$23,A6)</f>
+        <f>COUNTIF(Acompanhamento!$E$8:$E$24,A6)</f>
         <v/>
       </c>
       <c r="C6" s="18">
-        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A6),"")</f>
+        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A6),"")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$23,Acompanhamento!$E$8:$E$23,A6)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A6),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$24,Acompanhamento!$E$8:$E$24,A6)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A6),"")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A6)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A6),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A6)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A6),"")</f>
         <v/>
       </c>
       <c r="F6" s="18">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A6),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A6),"")</f>
         <v/>
       </c>
     </row>
@@ -1637,23 +1684,23 @@
         </is>
       </c>
       <c r="B7" s="17">
-        <f>COUNTIF(Acompanhamento!$E$8:$E$23,A7)</f>
+        <f>COUNTIF(Acompanhamento!$E$8:$E$24,A7)</f>
         <v/>
       </c>
       <c r="C7" s="18">
-        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A7),"")</f>
+        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A7),"")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$23,Acompanhamento!$E$8:$E$23,A7)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A7),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$24,Acompanhamento!$E$8:$E$24,A7)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A7),"")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A7)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A7),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A7)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A7),"")</f>
         <v/>
       </c>
       <c r="F7" s="18">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A7),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A7),"")</f>
         <v/>
       </c>
     </row>
@@ -1664,23 +1711,23 @@
         </is>
       </c>
       <c r="B8" s="17">
-        <f>COUNTIF(Acompanhamento!$E$8:$E$23,A8)</f>
+        <f>COUNTIF(Acompanhamento!$E$8:$E$24,A8)</f>
         <v/>
       </c>
       <c r="C8" s="18">
-        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A8),"")</f>
+        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A8),"")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$23,Acompanhamento!$E$8:$E$23,A8)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A8),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$24,Acompanhamento!$E$8:$E$24,A8)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A8),"")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A8)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A8),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A8)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A8),"")</f>
         <v/>
       </c>
       <c r="F8" s="18">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A8),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A8),"")</f>
         <v/>
       </c>
     </row>
@@ -1691,23 +1738,23 @@
         </is>
       </c>
       <c r="B9" s="17">
-        <f>COUNTIF(Acompanhamento!$E$8:$E$23,A9)</f>
+        <f>COUNTIF(Acompanhamento!$E$8:$E$24,A9)</f>
         <v/>
       </c>
       <c r="C9" s="18">
-        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A9),"")</f>
+        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A9),"")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$23,Acompanhamento!$E$8:$E$23,A9)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A9),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$24,Acompanhamento!$E$8:$E$24,A9)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A9),"")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A9)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A9),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A9)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A9),"")</f>
         <v/>
       </c>
       <c r="F9" s="18">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A9),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A9),"")</f>
         <v/>
       </c>
     </row>
@@ -1718,23 +1765,23 @@
         </is>
       </c>
       <c r="B10" s="17">
-        <f>COUNTIF(Acompanhamento!$E$8:$E$23,A10)</f>
+        <f>COUNTIF(Acompanhamento!$E$8:$E$24,A10)</f>
         <v/>
       </c>
       <c r="C10" s="18">
-        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A10),"")</f>
+        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A10),"")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$23,Acompanhamento!$E$8:$E$23,A10)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A10),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$24,Acompanhamento!$E$8:$E$24,A10)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A10),"")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A10)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A10),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A10)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A10),"")</f>
         <v/>
       </c>
       <c r="F10" s="18">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A10),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A10),"")</f>
         <v/>
       </c>
     </row>
@@ -1745,23 +1792,23 @@
         </is>
       </c>
       <c r="B11" s="17">
-        <f>COUNTIF(Acompanhamento!$E$8:$E$23,A11)</f>
+        <f>COUNTIF(Acompanhamento!$E$8:$E$24,A11)</f>
         <v/>
       </c>
       <c r="C11" s="18">
-        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A11),"")</f>
+        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A11),"")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$23,Acompanhamento!$E$8:$E$23,A11)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A11),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$24,Acompanhamento!$E$8:$E$24,A11)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A11),"")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A11)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A11),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A11)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A11),"")</f>
         <v/>
       </c>
       <c r="F11" s="18">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A11),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A11),"")</f>
         <v/>
       </c>
     </row>
@@ -1772,23 +1819,50 @@
         </is>
       </c>
       <c r="B12" s="17">
-        <f>COUNTIF(Acompanhamento!$E$8:$E$23,A12)</f>
+        <f>COUNTIF(Acompanhamento!$E$8:$E$24,A12)</f>
         <v/>
       </c>
       <c r="C12" s="18">
-        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A12),"")</f>
+        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A12),"")</f>
         <v/>
       </c>
       <c r="D12" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$23,Acompanhamento!$E$8:$E$23,A12)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A12),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$24,Acompanhamento!$E$8:$E$24,A12)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A12),"")</f>
         <v/>
       </c>
       <c r="E12" s="12">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A12)/SUMIFS(Acompanhamento!$G$8:$G$23,Acompanhamento!$E$8:$E$23,A12),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A12)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A12),"")</f>
         <v/>
       </c>
       <c r="F12" s="18">
-        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$23,Acompanhamento!$E$8:$E$23,A12),"")</f>
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Extra</t>
+        </is>
+      </c>
+      <c r="B13" s="17">
+        <f>COUNTIF(Acompanhamento!$E$8:$E$24,A13)</f>
+        <v/>
+      </c>
+      <c r="C13" s="18">
+        <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A13),"")</f>
+        <v/>
+      </c>
+      <c r="D13" s="12">
+        <f>IFERROR(SUMIFS(Acompanhamento!$H$8:$H$24,Acompanhamento!$E$8:$E$24,A13)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A13),"")</f>
+        <v/>
+      </c>
+      <c r="E13" s="12">
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A13)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A13),"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="18">
+        <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A13),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Lancar os dados reais do primeiro post publicado
Acrescenta a via de lancamento manual em dados/manual.json, contraparte do
coletor automatico enquanto a API nao esta ligada. A planilha passa a usar a
data real de publicacao quando ela existe, em vez da data derivada da grade,
e ordena as linhas por ela.

Dados do card de farinha, publicado em 20/08 e lido em 26/08: 2.769 contas
alcancadas, 20 salvamentos, 27 compartilhamentos, 3 comentarios, 41 visitas
ao perfil e 9 novos seguidores.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rs5hehAPo3WmcKFkRQTrtS
</commit_message>
<xml_diff>
--- a/analise/acompanhamento.xlsx
+++ b/analise/acompanhamento.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="dd/mm"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,6 +69,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF8A8578"/>
       <sz val="10"/>
     </font>
     <font>
@@ -127,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,9 +145,11 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,11 +157,10 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -699,36 +705,47 @@
       <c r="A8" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B8" s="10">
-        <f>$C$4+0</f>
-        <v/>
+      <c r="B8" s="10" t="n">
+        <v>46254</v>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Ter</t>
+          <t>Qui</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>65% de hidratação</t>
+          <t>Farinha importada</t>
         </is>
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>O Porquê do Número</t>
+          <t>Opinião Impopular</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>Carrossel</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="11" t="n"/>
-      <c r="I8" s="11" t="n"/>
-      <c r="J8" s="11" t="n"/>
-      <c r="K8" s="11" t="n"/>
-      <c r="L8" s="11" t="n"/>
+          <t>Card/Reels</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>2769</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>27</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="K8" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="L8" s="11" t="n">
+        <v>9</v>
+      </c>
       <c r="M8" s="12">
         <f>IFERROR(H8/G8,"")</f>
         <v/>
@@ -746,36 +763,36 @@
       <c r="A9" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="10">
-        <f>$C$4+1</f>
+      <c r="B9" s="13">
+        <f>$C$4+0</f>
         <v/>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Qua</t>
+          <t>Ter</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Pala e Pinsa, teglia e contemporânea</t>
+          <t>65% de hidratação</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Extra</t>
+          <t>O Porquê do Número</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Reels</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="n"/>
-      <c r="H9" s="11" t="n"/>
-      <c r="I9" s="11" t="n"/>
-      <c r="J9" s="11" t="n"/>
-      <c r="K9" s="11" t="n"/>
-      <c r="L9" s="11" t="n"/>
+          <t>Carrossel</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="n"/>
+      <c r="H9" s="14" t="n"/>
+      <c r="I9" s="14" t="n"/>
+      <c r="J9" s="14" t="n"/>
+      <c r="K9" s="14" t="n"/>
+      <c r="L9" s="14" t="n"/>
       <c r="M9" s="12">
         <f>IFERROR(H9/G9,"")</f>
         <v/>
@@ -793,36 +810,35 @@
       <c r="A10" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="10">
-        <f>$C$4+2</f>
-        <v/>
+      <c r="B10" s="10" t="n">
+        <v>46260</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Qui</t>
+          <t>Qua</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Farinha importada</t>
+          <t>Pala e Pinsa, teglia e contemporânea</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Opinião Impopular</t>
+          <t>Extra</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Card/Reels</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="n"/>
-      <c r="H10" s="11" t="n"/>
-      <c r="I10" s="11" t="n"/>
-      <c r="J10" s="11" t="n"/>
-      <c r="K10" s="11" t="n"/>
-      <c r="L10" s="11" t="n"/>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n"/>
+      <c r="H10" s="14" t="n"/>
+      <c r="I10" s="14" t="n"/>
+      <c r="J10" s="14" t="n"/>
+      <c r="K10" s="14" t="n"/>
+      <c r="L10" s="14" t="n"/>
       <c r="M10" s="12">
         <f>IFERROR(H10/G10,"")</f>
         <v/>
@@ -840,7 +856,7 @@
       <c r="A11" s="9" t="n">
         <v>4</v>
       </c>
-      <c r="B11" s="10">
+      <c r="B11" s="13">
         <f>$C$4+4</f>
         <v/>
       </c>
@@ -864,12 +880,12 @@
           <t>Foto</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n"/>
-      <c r="H11" s="11" t="n"/>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="11" t="n"/>
-      <c r="K11" s="11" t="n"/>
-      <c r="L11" s="11" t="n"/>
+      <c r="G11" s="14" t="n"/>
+      <c r="H11" s="14" t="n"/>
+      <c r="I11" s="14" t="n"/>
+      <c r="J11" s="14" t="n"/>
+      <c r="K11" s="14" t="n"/>
+      <c r="L11" s="14" t="n"/>
       <c r="M11" s="12">
         <f>IFERROR(H11/G11,"")</f>
         <v/>
@@ -887,7 +903,7 @@
       <c r="A12" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="13">
         <f>$C$4+5</f>
         <v/>
       </c>
@@ -911,12 +927,12 @@
           <t>Reels</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n"/>
-      <c r="H12" s="11" t="n"/>
-      <c r="I12" s="11" t="n"/>
-      <c r="J12" s="11" t="n"/>
-      <c r="K12" s="11" t="n"/>
-      <c r="L12" s="11" t="n"/>
+      <c r="G12" s="14" t="n"/>
+      <c r="H12" s="14" t="n"/>
+      <c r="I12" s="14" t="n"/>
+      <c r="J12" s="14" t="n"/>
+      <c r="K12" s="14" t="n"/>
+      <c r="L12" s="14" t="n"/>
       <c r="M12" s="12">
         <f>IFERROR(H12/G12,"")</f>
         <v/>
@@ -934,7 +950,7 @@
       <c r="A13" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B13" s="10">
+      <c r="B13" s="13">
         <f>$C$4+7</f>
         <v/>
       </c>
@@ -958,12 +974,12 @@
           <t>Carrossel</t>
         </is>
       </c>
-      <c r="G13" s="11" t="n"/>
-      <c r="H13" s="11" t="n"/>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n"/>
-      <c r="L13" s="11" t="n"/>
+      <c r="G13" s="14" t="n"/>
+      <c r="H13" s="14" t="n"/>
+      <c r="I13" s="14" t="n"/>
+      <c r="J13" s="14" t="n"/>
+      <c r="K13" s="14" t="n"/>
+      <c r="L13" s="14" t="n"/>
       <c r="M13" s="12">
         <f>IFERROR(H13/G13,"")</f>
         <v/>
@@ -981,7 +997,7 @@
       <c r="A14" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B14" s="10">
+      <c r="B14" s="13">
         <f>$C$4+9</f>
         <v/>
       </c>
@@ -1005,12 +1021,12 @@
           <t>Carrossel</t>
         </is>
       </c>
-      <c r="G14" s="11" t="n"/>
-      <c r="H14" s="11" t="n"/>
-      <c r="I14" s="11" t="n"/>
-      <c r="J14" s="11" t="n"/>
-      <c r="K14" s="11" t="n"/>
-      <c r="L14" s="11" t="n"/>
+      <c r="G14" s="14" t="n"/>
+      <c r="H14" s="14" t="n"/>
+      <c r="I14" s="14" t="n"/>
+      <c r="J14" s="14" t="n"/>
+      <c r="K14" s="14" t="n"/>
+      <c r="L14" s="14" t="n"/>
       <c r="M14" s="12">
         <f>IFERROR(H14/G14,"")</f>
         <v/>
@@ -1028,7 +1044,7 @@
       <c r="A15" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B15" s="10">
+      <c r="B15" s="13">
         <f>$C$4+11</f>
         <v/>
       </c>
@@ -1052,12 +1068,12 @@
           <t>Carrossel</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n"/>
-      <c r="H15" s="11" t="n"/>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="11" t="n"/>
-      <c r="K15" s="11" t="n"/>
-      <c r="L15" s="11" t="n"/>
+      <c r="G15" s="14" t="n"/>
+      <c r="H15" s="14" t="n"/>
+      <c r="I15" s="14" t="n"/>
+      <c r="J15" s="14" t="n"/>
+      <c r="K15" s="14" t="n"/>
+      <c r="L15" s="14" t="n"/>
       <c r="M15" s="12">
         <f>IFERROR(H15/G15,"")</f>
         <v/>
@@ -1075,7 +1091,7 @@
       <c r="A16" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="10">
+      <c r="B16" s="13">
         <f>$C$4+12</f>
         <v/>
       </c>
@@ -1099,12 +1115,12 @@
           <t>Reels</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n"/>
-      <c r="H16" s="11" t="n"/>
-      <c r="I16" s="11" t="n"/>
-      <c r="J16" s="11" t="n"/>
-      <c r="K16" s="11" t="n"/>
-      <c r="L16" s="11" t="n"/>
+      <c r="G16" s="14" t="n"/>
+      <c r="H16" s="14" t="n"/>
+      <c r="I16" s="14" t="n"/>
+      <c r="J16" s="14" t="n"/>
+      <c r="K16" s="14" t="n"/>
+      <c r="L16" s="14" t="n"/>
       <c r="M16" s="12">
         <f>IFERROR(H16/G16,"")</f>
         <v/>
@@ -1122,7 +1138,7 @@
       <c r="A17" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="10">
+      <c r="B17" s="13">
         <f>$C$4+14</f>
         <v/>
       </c>
@@ -1146,12 +1162,12 @@
           <t>Carrossel</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n"/>
-      <c r="H17" s="11" t="n"/>
-      <c r="I17" s="11" t="n"/>
-      <c r="J17" s="11" t="n"/>
-      <c r="K17" s="11" t="n"/>
-      <c r="L17" s="11" t="n"/>
+      <c r="G17" s="14" t="n"/>
+      <c r="H17" s="14" t="n"/>
+      <c r="I17" s="14" t="n"/>
+      <c r="J17" s="14" t="n"/>
+      <c r="K17" s="14" t="n"/>
+      <c r="L17" s="14" t="n"/>
       <c r="M17" s="12">
         <f>IFERROR(H17/G17,"")</f>
         <v/>
@@ -1169,7 +1185,7 @@
       <c r="A18" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="13">
         <f>$C$4+16</f>
         <v/>
       </c>
@@ -1193,12 +1209,12 @@
           <t>Card/Reels</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n"/>
-      <c r="H18" s="11" t="n"/>
-      <c r="I18" s="11" t="n"/>
-      <c r="J18" s="11" t="n"/>
-      <c r="K18" s="11" t="n"/>
-      <c r="L18" s="11" t="n"/>
+      <c r="G18" s="14" t="n"/>
+      <c r="H18" s="14" t="n"/>
+      <c r="I18" s="14" t="n"/>
+      <c r="J18" s="14" t="n"/>
+      <c r="K18" s="14" t="n"/>
+      <c r="L18" s="14" t="n"/>
       <c r="M18" s="12">
         <f>IFERROR(H18/G18,"")</f>
         <v/>
@@ -1216,7 +1232,7 @@
       <c r="A19" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="10">
+      <c r="B19" s="13">
         <f>$C$4+18</f>
         <v/>
       </c>
@@ -1240,12 +1256,12 @@
           <t>Reels</t>
         </is>
       </c>
-      <c r="G19" s="11" t="n"/>
-      <c r="H19" s="11" t="n"/>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="11" t="n"/>
-      <c r="K19" s="11" t="n"/>
-      <c r="L19" s="11" t="n"/>
+      <c r="G19" s="14" t="n"/>
+      <c r="H19" s="14" t="n"/>
+      <c r="I19" s="14" t="n"/>
+      <c r="J19" s="14" t="n"/>
+      <c r="K19" s="14" t="n"/>
+      <c r="L19" s="14" t="n"/>
       <c r="M19" s="12">
         <f>IFERROR(H19/G19,"")</f>
         <v/>
@@ -1263,7 +1279,7 @@
       <c r="A20" s="9" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="10">
+      <c r="B20" s="13">
         <f>$C$4+19</f>
         <v/>
       </c>
@@ -1287,12 +1303,12 @@
           <t>Reels</t>
         </is>
       </c>
-      <c r="G20" s="11" t="n"/>
-      <c r="H20" s="11" t="n"/>
-      <c r="I20" s="11" t="n"/>
-      <c r="J20" s="11" t="n"/>
-      <c r="K20" s="11" t="n"/>
-      <c r="L20" s="11" t="n"/>
+      <c r="G20" s="14" t="n"/>
+      <c r="H20" s="14" t="n"/>
+      <c r="I20" s="14" t="n"/>
+      <c r="J20" s="14" t="n"/>
+      <c r="K20" s="14" t="n"/>
+      <c r="L20" s="14" t="n"/>
       <c r="M20" s="12">
         <f>IFERROR(H20/G20,"")</f>
         <v/>
@@ -1310,7 +1326,7 @@
       <c r="A21" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="10">
+      <c r="B21" s="13">
         <f>$C$4+21</f>
         <v/>
       </c>
@@ -1334,12 +1350,12 @@
           <t>Carrossel</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n"/>
-      <c r="H21" s="11" t="n"/>
-      <c r="I21" s="11" t="n"/>
-      <c r="J21" s="11" t="n"/>
-      <c r="K21" s="11" t="n"/>
-      <c r="L21" s="11" t="n"/>
+      <c r="G21" s="14" t="n"/>
+      <c r="H21" s="14" t="n"/>
+      <c r="I21" s="14" t="n"/>
+      <c r="J21" s="14" t="n"/>
+      <c r="K21" s="14" t="n"/>
+      <c r="L21" s="14" t="n"/>
       <c r="M21" s="12">
         <f>IFERROR(H21/G21,"")</f>
         <v/>
@@ -1357,7 +1373,7 @@
       <c r="A22" s="9" t="n">
         <v>15</v>
       </c>
-      <c r="B22" s="10">
+      <c r="B22" s="13">
         <f>$C$4+23</f>
         <v/>
       </c>
@@ -1381,12 +1397,12 @@
           <t>Carrossel</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n"/>
-      <c r="H22" s="11" t="n"/>
-      <c r="I22" s="11" t="n"/>
-      <c r="J22" s="11" t="n"/>
-      <c r="K22" s="11" t="n"/>
-      <c r="L22" s="11" t="n"/>
+      <c r="G22" s="14" t="n"/>
+      <c r="H22" s="14" t="n"/>
+      <c r="I22" s="14" t="n"/>
+      <c r="J22" s="14" t="n"/>
+      <c r="K22" s="14" t="n"/>
+      <c r="L22" s="14" t="n"/>
       <c r="M22" s="12">
         <f>IFERROR(H22/G22,"")</f>
         <v/>
@@ -1404,7 +1420,7 @@
       <c r="A23" s="9" t="n">
         <v>16</v>
       </c>
-      <c r="B23" s="10">
+      <c r="B23" s="13">
         <f>$C$4+25</f>
         <v/>
       </c>
@@ -1428,12 +1444,12 @@
           <t>Carrossel</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n"/>
-      <c r="H23" s="11" t="n"/>
-      <c r="I23" s="11" t="n"/>
-      <c r="J23" s="11" t="n"/>
-      <c r="K23" s="11" t="n"/>
-      <c r="L23" s="11" t="n"/>
+      <c r="G23" s="14" t="n"/>
+      <c r="H23" s="14" t="n"/>
+      <c r="I23" s="14" t="n"/>
+      <c r="J23" s="14" t="n"/>
+      <c r="K23" s="14" t="n"/>
+      <c r="L23" s="14" t="n"/>
       <c r="M23" s="12">
         <f>IFERROR(H23/G23,"")</f>
         <v/>
@@ -1451,7 +1467,7 @@
       <c r="A24" s="9" t="n">
         <v>17</v>
       </c>
-      <c r="B24" s="10">
+      <c r="B24" s="13">
         <f>$C$4+26</f>
         <v/>
       </c>
@@ -1475,12 +1491,12 @@
           <t>Reels</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n"/>
-      <c r="H24" s="11" t="n"/>
-      <c r="I24" s="11" t="n"/>
-      <c r="J24" s="11" t="n"/>
-      <c r="K24" s="11" t="n"/>
-      <c r="L24" s="11" t="n"/>
+      <c r="G24" s="14" t="n"/>
+      <c r="H24" s="14" t="n"/>
+      <c r="I24" s="14" t="n"/>
+      <c r="J24" s="14" t="n"/>
+      <c r="K24" s="14" t="n"/>
+      <c r="L24" s="14" t="n"/>
       <c r="M24" s="12">
         <f>IFERROR(H24/G24,"")</f>
         <v/>
@@ -1500,39 +1516,39 @@
           <t>MÉDIA DO MÊS</t>
         </is>
       </c>
-      <c r="G26" s="13">
+      <c r="G26" s="15">
         <f>IFERROR(AVERAGE(G8:G24),"")</f>
         <v/>
       </c>
-      <c r="H26" s="13">
+      <c r="H26" s="15">
         <f>IFERROR(AVERAGE(H8:H24),"")</f>
         <v/>
       </c>
-      <c r="I26" s="13">
+      <c r="I26" s="15">
         <f>IFERROR(AVERAGE(I8:I24),"")</f>
         <v/>
       </c>
-      <c r="J26" s="13">
+      <c r="J26" s="15">
         <f>IFERROR(AVERAGE(J8:J24),"")</f>
         <v/>
       </c>
-      <c r="K26" s="13">
+      <c r="K26" s="15">
         <f>IFERROR(AVERAGE(K8:K24),"")</f>
         <v/>
       </c>
-      <c r="L26" s="13">
+      <c r="L26" s="15">
         <f>IFERROR(AVERAGE(L8:L24),"")</f>
         <v/>
       </c>
-      <c r="M26" s="14">
+      <c r="M26" s="16">
         <f>IFERROR(AVERAGE(M8:M24),"")</f>
         <v/>
       </c>
-      <c r="N26" s="14">
+      <c r="N26" s="16">
         <f>IFERROR(AVERAGE(N8:N24),"")</f>
         <v/>
       </c>
-      <c r="O26" s="14">
+      <c r="O26" s="16">
         <f>IFERROR(AVERAGE(O8:O24),"")</f>
         <v/>
       </c>
@@ -1546,7 +1562,7 @@
       <c r="L27" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="N27" s="15" t="n">
+      <c r="N27" s="17" t="n">
         <v>0.003</v>
       </c>
       <c r="O27" s="5" t="inlineStr">
@@ -1592,32 +1608,32 @@
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="18" t="inlineStr">
         <is>
           <t>Série</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="18" t="inlineStr">
         <is>
           <t>Posts</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Alcance médio</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Salv./alcance</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Segui./alcance</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Seguidores no total</t>
         </is>
@@ -1629,11 +1645,11 @@
           <t>O Porquê do Número</t>
         </is>
       </c>
-      <c r="B5" s="17">
+      <c r="B5" s="19">
         <f>COUNTIF(Acompanhamento!$E$8:$E$24,A5)</f>
         <v/>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="11">
         <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A5),"")</f>
         <v/>
       </c>
@@ -1645,7 +1661,7 @@
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A5)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A5),"")</f>
         <v/>
       </c>
-      <c r="F5" s="18">
+      <c r="F5" s="11">
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A5),"")</f>
         <v/>
       </c>
@@ -1656,11 +1672,11 @@
           <t>Opinião Impopular</t>
         </is>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="19">
         <f>COUNTIF(Acompanhamento!$E$8:$E$24,A6)</f>
         <v/>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="11">
         <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A6),"")</f>
         <v/>
       </c>
@@ -1672,7 +1688,7 @@
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A6)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A6),"")</f>
         <v/>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="11">
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A6),"")</f>
         <v/>
       </c>
@@ -1683,11 +1699,11 @@
           <t>Uma Variável</t>
         </is>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="19">
         <f>COUNTIF(Acompanhamento!$E$8:$E$24,A7)</f>
         <v/>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="11">
         <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A7),"")</f>
         <v/>
       </c>
@@ -1699,7 +1715,7 @@
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A7)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A7),"")</f>
         <v/>
       </c>
-      <c r="F7" s="18">
+      <c r="F7" s="11">
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A7),"")</f>
         <v/>
       </c>
@@ -1710,11 +1726,11 @@
           <t>O Porquê</t>
         </is>
       </c>
-      <c r="B8" s="17">
+      <c r="B8" s="19">
         <f>COUNTIF(Acompanhamento!$E$8:$E$24,A8)</f>
         <v/>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="11">
         <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A8),"")</f>
         <v/>
       </c>
@@ -1726,7 +1742,7 @@
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A8)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A8),"")</f>
         <v/>
       </c>
-      <c r="F8" s="18">
+      <c r="F8" s="11">
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A8),"")</f>
         <v/>
       </c>
@@ -1737,11 +1753,11 @@
           <t>Autoral</t>
         </is>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="19">
         <f>COUNTIF(Acompanhamento!$E$8:$E$24,A9)</f>
         <v/>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="11">
         <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A9),"")</f>
         <v/>
       </c>
@@ -1753,7 +1769,7 @@
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A9)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A9),"")</f>
         <v/>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="11">
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A9),"")</f>
         <v/>
       </c>
@@ -1764,11 +1780,11 @@
           <t>Bastidores</t>
         </is>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="19">
         <f>COUNTIF(Acompanhamento!$E$8:$E$24,A10)</f>
         <v/>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="11">
         <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A10),"")</f>
         <v/>
       </c>
@@ -1780,7 +1796,7 @@
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A10)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A10),"")</f>
         <v/>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="11">
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A10),"")</f>
         <v/>
       </c>
@@ -1791,11 +1807,11 @@
           <t>O Erro</t>
         </is>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="19">
         <f>COUNTIF(Acompanhamento!$E$8:$E$24,A11)</f>
         <v/>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="11">
         <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A11),"")</f>
         <v/>
       </c>
@@ -1807,7 +1823,7 @@
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A11)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A11),"")</f>
         <v/>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="11">
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A11),"")</f>
         <v/>
       </c>
@@ -1818,11 +1834,11 @@
           <t>Formação</t>
         </is>
       </c>
-      <c r="B12" s="17">
+      <c r="B12" s="19">
         <f>COUNTIF(Acompanhamento!$E$8:$E$24,A12)</f>
         <v/>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="11">
         <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A12),"")</f>
         <v/>
       </c>
@@ -1834,7 +1850,7 @@
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A12)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A12),"")</f>
         <v/>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="11">
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A12),"")</f>
         <v/>
       </c>
@@ -1845,11 +1861,11 @@
           <t>Extra</t>
         </is>
       </c>
-      <c r="B13" s="17">
+      <c r="B13" s="19">
         <f>COUNTIF(Acompanhamento!$E$8:$E$24,A13)</f>
         <v/>
       </c>
-      <c r="C13" s="18">
+      <c r="C13" s="11">
         <f>IFERROR(AVERAGEIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A13),"")</f>
         <v/>
       </c>
@@ -1861,7 +1877,7 @@
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A13)/SUMIFS(Acompanhamento!$G$8:$G$24,Acompanhamento!$E$8:$E$24,A13),"")</f>
         <v/>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="11">
         <f>IFERROR(SUMIFS(Acompanhamento!$L$8:$L$24,Acompanhamento!$E$8:$E$24,A13),"")</f>
         <v/>
       </c>
@@ -1892,147 +1908,147 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="19" t="n"/>
+      <c r="B3" s="20" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Salv./alcance</t>
         </is>
       </c>
-      <c r="B4" s="21" t="inlineStr">
+      <c r="B4" s="22" t="inlineStr">
         <is>
           <t>O indicador mais importante aqui. Conteúdo educativo bom é salvo, e salvamento é o sinal mais forte que existe pro algoritmo reentregar.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Abaixo de 1%: o post informou mas não foi útil o suficiente pra guardar.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="21" t="inlineStr">
+      <c r="B6" s="22" t="inlineStr">
         <is>
           <t>1% a 3%: bom. É a faixa que sustenta crescimento.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="21" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>Acima de 3%: repita o formato. Achou uma veia.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="19" t="n"/>
+      <c r="B8" s="20" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="21" t="inlineStr">
         <is>
           <t>Segui./alcance</t>
         </is>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="22" t="inlineStr">
         <is>
           <t>A conversão. É o número que responde se o post fez a pessoa querer ficar.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="21" t="inlineStr">
+      <c r="B10" s="22" t="inlineStr">
         <is>
           <t>Hoje o perfil está abaixo de 0,3%, calculado sobre 49.900 views e o histórico de 14 seguidores por post.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="21" t="inlineStr">
+      <c r="B11" s="22" t="inlineStr">
         <is>
           <t>A meta dos 30 dias é dobrar isso. Chegando em 1% com o mesmo alcance de hoje, são cerca de 500 seguidores por mês.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="19" t="n"/>
+      <c r="B12" s="20" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Visitas/alcance</t>
         </is>
       </c>
-      <c r="B13" s="21" t="inlineStr">
+      <c r="B13" s="22" t="inlineStr">
         <is>
           <t>Intenção. A pessoa viu o post e foi conferir o perfil.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="21" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>Visita alta com conversão baixa significa que o post funciona e o perfil não segura. Aí o problema é bio e fixados, não conteúdo.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="19" t="n"/>
+      <c r="B15" s="20" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Comentários</t>
         </is>
       </c>
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>Não entra no cálculo de retenção, mas é o que mais empurra alcance. Espere Opinião Impopular liderar aqui.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="19" t="n"/>
+      <c r="B17" s="20" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>Onde achar</t>
         </is>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="22" t="inlineStr">
         <is>
           <t>Instagram, abre o post, toca em Ver insights. Reels mostra também tempo médio de visualização, que vale anotar à parte.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="19" t="n"/>
+      <c r="B19" s="20" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Quando analisar</t>
         </is>
       </c>
-      <c r="B20" s="21" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>Espere 72 horas depois de publicar antes de anotar, porque o post continua rodando. Compare só depois de 8 posts, que é quando o padrão aparece.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="19" t="n"/>
+      <c r="B21" s="20" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="A22" s="21" t="inlineStr">
         <is>
           <t>O que a análise decide</t>
         </is>
       </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="B22" s="22" t="inlineStr">
         <is>
           <t>No fim das 4 semanas, a aba Por série mostra qual formato retém mais. O mês seguinte se escreve em cima dessa resposta, não de palpite.</t>
         </is>

</xml_diff>

<commit_message>
Lancar os dados do Reels Pala e Pinsa
Alcance de 2.705 contas, 3.633 visualizacoes, 13s de tempo medio num video
de 53s, 41,6% de pulados, 66,2% de nao seguidores. Sete salvamentos, cinco
compartilhamentos, nove comentarios, oito visitas ao perfil e dois novos
seguidores.

Registra tambem quantas hashtags cada post levou e se tinha CTA de
comentario, que sao as duas variaveis em teste.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rs5hehAPo3WmcKFkRQTrtS
</commit_message>
<xml_diff>
--- a/analise/acompanhamento.xlsx
+++ b/analise/acompanhamento.xlsx
@@ -833,12 +833,24 @@
           <t>Reels</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n"/>
-      <c r="H10" s="14" t="n"/>
-      <c r="I10" s="14" t="n"/>
-      <c r="J10" s="14" t="n"/>
-      <c r="K10" s="14" t="n"/>
-      <c r="L10" s="14" t="n"/>
+      <c r="G10" s="11" t="n">
+        <v>2705</v>
+      </c>
+      <c r="H10" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="I10" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="K10" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L10" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="M10" s="12">
         <f>IFERROR(H10/G10,"")</f>
         <v/>

</xml_diff>

<commit_message>
Marcar o carrossel de 75% como publicado em 01/09
O post foi agendado para 01/09 as 14h30, com sete imagens e a foto real do
corte na posicao cinco. Fica sem numeros ate a Routine cobrar na segunda
14/09, quando ele tera 13 dias.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rs5hehAPo3WmcKFkRQTrtS
</commit_message>
<xml_diff>
--- a/analise/acompanhamento.xlsx
+++ b/analise/acompanhamento.xlsx
@@ -763,36 +763,47 @@
       <c r="A9" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B9" s="13">
-        <f>$C$4+0</f>
-        <v/>
+      <c r="B9" s="10" t="n">
+        <v>46260</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Ter</t>
+          <t>Qua</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>75% de hidratação</t>
+          <t>Pala e Pinsa, teglia e contemporânea</t>
         </is>
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>O Porquê do Número</t>
+          <t>Extra</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Carrossel</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
-      <c r="I9" s="14" t="n"/>
-      <c r="J9" s="14" t="n"/>
-      <c r="K9" s="14" t="n"/>
-      <c r="L9" s="14" t="n"/>
+          <t>Reels</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>2705</v>
+      </c>
+      <c r="H9" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="I9" s="11" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="K9" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="L9" s="11" t="n">
+        <v>2</v>
+      </c>
       <c r="M9" s="12">
         <f>IFERROR(H9/G9,"")</f>
         <v/>
@@ -810,47 +821,36 @@
       <c r="A10" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B10" s="10" t="n">
-        <v>46260</v>
+      <c r="B10" s="13">
+        <f>$C$4+4</f>
+        <v/>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Qua</t>
+          <t>Sáb</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Pala e Pinsa, teglia e contemporânea</t>
+          <t>Criação autoral</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Extra</t>
+          <t>Autoral</t>
         </is>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
-          <t>Reels</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>2705</v>
-      </c>
-      <c r="H10" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="I10" s="11" t="n">
-        <v>5</v>
-      </c>
-      <c r="J10" s="11" t="n">
-        <v>9</v>
-      </c>
-      <c r="K10" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="L10" s="11" t="n">
-        <v>2</v>
-      </c>
+          <t>Foto</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n"/>
+      <c r="H10" s="14" t="n"/>
+      <c r="I10" s="14" t="n"/>
+      <c r="J10" s="14" t="n"/>
+      <c r="K10" s="14" t="n"/>
+      <c r="L10" s="14" t="n"/>
       <c r="M10" s="12">
         <f>IFERROR(H10/G10,"")</f>
         <v/>
@@ -869,27 +869,27 @@
         <v>4</v>
       </c>
       <c r="B11" s="13">
-        <f>$C$4+4</f>
+        <f>$C$4+5</f>
         <v/>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Sáb</t>
+          <t>Dom</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Criação autoral</t>
+          <t>Ponto de véu</t>
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Autoral</t>
+          <t>O Porquê</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Foto</t>
+          <t>Reels</t>
         </is>
       </c>
       <c r="G11" s="14" t="n"/>
@@ -915,28 +915,27 @@
       <c r="A12" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B12" s="13">
-        <f>$C$4+5</f>
-        <v/>
+      <c r="B12" s="10" t="n">
+        <v>46266</v>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Dom</t>
+          <t>Ter</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Ponto de véu</t>
+          <t>75% de hidratação</t>
         </is>
       </c>
       <c r="E12" s="9" t="inlineStr">
         <is>
-          <t>O Porquê</t>
+          <t>O Porquê do Número</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Reels</t>
+          <t>Carrossel</t>
         </is>
       </c>
       <c r="G12" s="14" t="n"/>

</xml_diff>